<commit_message>
save local before merging master
</commit_message>
<xml_diff>
--- a/src/test/resources/Dietician_Exceldata.xlsx
+++ b/src/test/resources/Dietician_Exceldata.xlsx
@@ -1,23 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="6" rupBuild="4505"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rresh\eclipse-workspace\Team03Dietician_Project\src\test\resources\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{159B1A42-3D0D-4491-B23C-DE83C2A60C12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="19392" windowHeight="10392" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="login" sheetId="1" r:id="rId1"/>
+    <sheet name="editPatientSheetName" sheetId="2" r:id="rId2"/>
+    <sheet name="deletePatientSheetName" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+  <calcPr calcId="124519"/>
+  <extLst xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -25,16 +21,37 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>scenario_type</t>
   </si>
+  <si>
+    <t>Scenario_Type</t>
+  </si>
+  <si>
+    <t>firstName</t>
+  </si>
+  <si>
+    <t>lastName</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>contactNo</t>
+  </si>
+  <si>
+    <t>allergies</t>
+  </si>
+  <si>
+    <t>foodPreference</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -125,7 +142,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -160,7 +177,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -337,21 +354,21 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="14.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:1">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -359,4 +376,52 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="5" max="5" width="11" customWidth="1"/>
+    <col min="7" max="7" width="13.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
updated works POM editsteps
</commit_message>
<xml_diff>
--- a/src/test/resources/Dietician_Exceldata.xlsx
+++ b/src/test/resources/Dietician_Exceldata.xlsx
@@ -1,18 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr/>
+  <bookViews>
+    <workbookView xWindow="588" yWindow="516" windowWidth="15996" windowHeight="5244" activeTab="2"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="login" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="AddPatient" sheetId="2" r:id="rId6"/>
+    <sheet name="login" sheetId="1" r:id="rId1"/>
+    <sheet name="AddPatient" sheetId="2" r:id="rId2"/>
+    <sheet name="editPatient" sheetId="3" r:id="rId3"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="92">
   <si>
     <t>scenario_type</t>
   </si>
@@ -70,20 +74,26 @@
   <si>
     <r>
       <rPr>
+        <sz val="11"/>
         <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
       </rPr>
       <t>abc</t>
     </r>
     <r>
       <rPr>
+        <u/>
+        <sz val="11"/>
         <color rgb="FF1155CC"/>
-        <u/>
+        <rFont val="Calibri"/>
       </rPr>
       <t>@test.c</t>
     </r>
     <r>
       <rPr>
+        <sz val="11"/>
         <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
       </rPr>
       <t>om</t>
     </r>
@@ -112,8 +122,10 @@
   <si>
     <r>
       <rPr>
+        <u/>
+        <sz val="11"/>
         <color rgb="FF1155CC"/>
-        <u/>
+        <rFont val="Calibri"/>
       </rPr>
       <t>jane@test.com</t>
     </r>
@@ -129,40 +141,267 @@
   </si>
   <si>
     <t>largefile</t>
+  </si>
+  <si>
+    <t>ValidFirst Name</t>
+  </si>
+  <si>
+    <t>ValidLast Name</t>
+  </si>
+  <si>
+    <t>ValidEmail</t>
+  </si>
+  <si>
+    <t>ValidContact No</t>
+  </si>
+  <si>
+    <t>ValidWeight</t>
+  </si>
+  <si>
+    <t>ValidHeight</t>
+  </si>
+  <si>
+    <t>ValidTemperature</t>
+  </si>
+  <si>
+    <t>ValidSP</t>
+  </si>
+  <si>
+    <t>ValidDP</t>
+  </si>
+  <si>
+    <t>Valid SP and DP</t>
+  </si>
+  <si>
+    <t>ValidDate</t>
+  </si>
+  <si>
+    <t>teamab</t>
+  </si>
+  <si>
+    <t>proph</t>
+  </si>
+  <si>
+    <t>ab@gmail.com</t>
+  </si>
+  <si>
+    <t>FirstName with numeric</t>
+  </si>
+  <si>
+    <t>ab234</t>
+  </si>
+  <si>
+    <t>FirstName with spl Char and Numeric</t>
+  </si>
+  <si>
+    <t>ab234!%</t>
+  </si>
+  <si>
+    <t>FirstName with spl Char</t>
+  </si>
+  <si>
+    <t>ab%#</t>
+  </si>
+  <si>
+    <t>LastName with numeric</t>
+  </si>
+  <si>
+    <t>LastName with spl Char and Numeric</t>
+  </si>
+  <si>
+    <t>LastName with spl Char</t>
+  </si>
+  <si>
+    <t>Email with invalid format</t>
+  </si>
+  <si>
+    <t>Email with spl char</t>
+  </si>
+  <si>
+    <t>Email with missing @</t>
+  </si>
+  <si>
+    <t>Email with empty field</t>
+  </si>
+  <si>
+    <t>ContactNumber with alphabets</t>
+  </si>
+  <si>
+    <t>ContactNumber with spl Char</t>
+  </si>
+  <si>
+    <t>ContactNumber with less Digits</t>
+  </si>
+  <si>
+    <t>ContactNumber as Empty</t>
+  </si>
+  <si>
+    <t>Weight with Alphabets</t>
+  </si>
+  <si>
+    <t>Weight with spl char</t>
+  </si>
+  <si>
+    <t>Height with Alphabets</t>
+  </si>
+  <si>
+    <t>Height with spl char</t>
+  </si>
+  <si>
+    <t>Temp with Alphabets</t>
+  </si>
+  <si>
+    <t>Temp with spl char</t>
+  </si>
+  <si>
+    <t>SP with spl char</t>
+  </si>
+  <si>
+    <t>SP with Alphabets</t>
+  </si>
+  <si>
+    <t>Only SP</t>
+  </si>
+  <si>
+    <t>DP with spl char</t>
+  </si>
+  <si>
+    <t>DP with Alphabets</t>
+  </si>
+  <si>
+    <t>only DP</t>
+  </si>
+  <si>
+    <t>pro23</t>
+  </si>
+  <si>
+    <t>pro23#%</t>
+  </si>
+  <si>
+    <t>pro#!</t>
+  </si>
+  <si>
+    <t>sdgmail@com</t>
+  </si>
+  <si>
+    <t>ab##@gmail.com</t>
+  </si>
+  <si>
+    <t>abgmail.com</t>
+  </si>
+  <si>
+    <t>87945dfrdd</t>
+  </si>
+  <si>
+    <t>45364@#</t>
+  </si>
+  <si>
+    <t>5a</t>
+  </si>
+  <si>
+    <t>5#</t>
+  </si>
+  <si>
+    <t>155a</t>
+  </si>
+  <si>
+    <t>15!</t>
+  </si>
+  <si>
+    <t>99s</t>
+  </si>
+  <si>
+    <t>99!</t>
+  </si>
+  <si>
+    <t>94!</t>
+  </si>
+  <si>
+    <t>94a</t>
+  </si>
+  <si>
+    <t>78&amp;</t>
+  </si>
+  <si>
+    <t>78q</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="11">
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
       <u/>
+      <sz val="11"/>
       <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <u/>
+      <sz val="11"/>
       <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF1155CC"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -170,57 +409,57 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+  <cellStyleXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="15">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -410,40 +649,40 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:A1000"/>
+  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="14.71"/>
-    <col customWidth="1" min="2" max="26" width="8.71"/>
+    <col min="1" max="1" width="14.6640625" customWidth="1"/>
+    <col min="2" max="26" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.25" customHeight="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:1" ht="14.25" customHeight="1">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" ht="14.25" customHeight="1"/>
-    <row r="3" ht="14.25" customHeight="1"/>
-    <row r="4" ht="14.25" customHeight="1"/>
-    <row r="5" ht="14.25" customHeight="1"/>
-    <row r="6" ht="14.25" customHeight="1"/>
-    <row r="7" ht="14.25" customHeight="1"/>
-    <row r="8" ht="14.25" customHeight="1"/>
-    <row r="9" ht="14.25" customHeight="1"/>
-    <row r="10" ht="14.25" customHeight="1"/>
-    <row r="11" ht="14.25" customHeight="1"/>
-    <row r="12" ht="14.25" customHeight="1"/>
-    <row r="13" ht="14.25" customHeight="1"/>
-    <row r="14" ht="14.25" customHeight="1"/>
-    <row r="15" ht="14.25" customHeight="1"/>
-    <row r="16" ht="14.25" customHeight="1"/>
+    <row r="2" spans="1:1" ht="14.25" customHeight="1"/>
+    <row r="3" spans="1:1" ht="14.25" customHeight="1"/>
+    <row r="4" spans="1:1" ht="14.25" customHeight="1"/>
+    <row r="5" spans="1:1" ht="14.25" customHeight="1"/>
+    <row r="6" spans="1:1" ht="14.25" customHeight="1"/>
+    <row r="7" spans="1:1" ht="14.25" customHeight="1"/>
+    <row r="8" spans="1:1" ht="14.25" customHeight="1"/>
+    <row r="9" spans="1:1" ht="14.25" customHeight="1"/>
+    <row r="10" spans="1:1" ht="14.25" customHeight="1"/>
+    <row r="11" spans="1:1" ht="14.25" customHeight="1"/>
+    <row r="12" spans="1:1" ht="14.25" customHeight="1"/>
+    <row r="13" spans="1:1" ht="14.25" customHeight="1"/>
+    <row r="14" spans="1:1" ht="14.25" customHeight="1"/>
+    <row r="15" spans="1:1" ht="14.25" customHeight="1"/>
+    <row r="16" spans="1:1" ht="14.25" customHeight="1"/>
     <row r="17" ht="14.25" customHeight="1"/>
     <row r="18" ht="14.25" customHeight="1"/>
     <row r="19" ht="14.25" customHeight="1"/>
@@ -1429,166 +1668,526 @@
     <row r="999" ht="14.25" customHeight="1"/>
     <row r="1000" ht="14.25" customHeight="1"/>
   </sheetData>
-  <printOptions/>
-  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
-  <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
+  <pageSetup orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+  <dimension ref="A1:O3"/>
+  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:15">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:15">
+      <c r="A2" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E2" s="3">
-        <v>9.87654321E9</v>
-      </c>
-      <c r="F2" s="3" t="s">
+      <c r="E2" s="2">
+        <v>9876543210</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="I2" s="5">
-        <v>36537.0</v>
-      </c>
-      <c r="J2" s="3">
-        <v>70.0</v>
-      </c>
-      <c r="K2" s="3">
+      <c r="I2" s="4">
+        <v>36537</v>
+      </c>
+      <c r="J2" s="2">
+        <v>70</v>
+      </c>
+      <c r="K2" s="2">
         <v>5.5</v>
       </c>
-      <c r="L2" s="3">
-        <v>98.0</v>
-      </c>
-      <c r="M2" s="3">
-        <v>120.0</v>
-      </c>
-      <c r="N2" s="3">
-        <v>80.0</v>
-      </c>
-      <c r="O2" s="3" t="s">
+      <c r="L2" s="2">
+        <v>98</v>
+      </c>
+      <c r="M2" s="2">
+        <v>120</v>
+      </c>
+      <c r="N2" s="2">
+        <v>80</v>
+      </c>
+      <c r="O2" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="s">
+    <row r="3" spans="1:15">
+      <c r="A3" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="E3" s="3">
-        <v>1.23456789E9</v>
-      </c>
-      <c r="F3" s="3" t="s">
+      <c r="E3" s="2">
+        <v>1234567890</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="I3" s="5">
-        <v>34824.0</v>
-      </c>
-      <c r="J3" s="3">
-        <v>65.0</v>
-      </c>
-      <c r="K3" s="3">
+      <c r="I3" s="4">
+        <v>34824</v>
+      </c>
+      <c r="J3" s="2">
+        <v>65</v>
+      </c>
+      <c r="K3" s="2">
         <v>5.3</v>
       </c>
-      <c r="L3" s="3">
-        <v>100.0</v>
-      </c>
-      <c r="M3" s="3">
-        <v>130.0</v>
-      </c>
-      <c r="N3" s="3">
-        <v>85.0</v>
-      </c>
-      <c r="O3" s="3" t="s">
+      <c r="L3" s="2">
+        <v>100</v>
+      </c>
+      <c r="M3" s="2">
+        <v>130</v>
+      </c>
+      <c r="N3" s="2">
+        <v>85</v>
+      </c>
+      <c r="O3" s="2" t="s">
         <v>30</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="D2"/>
-    <hyperlink r:id="rId2" ref="D3"/>
+    <hyperlink ref="D2" r:id="rId1"/>
+    <hyperlink ref="D3" r:id="rId2"/>
   </hyperlinks>
-  <drawing r:id="rId3"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:O38"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="36.44140625" customWidth="1"/>
+    <col min="2" max="2" width="14.5546875" customWidth="1"/>
+    <col min="3" max="3" width="14.21875" customWidth="1"/>
+    <col min="4" max="4" width="14.6640625" customWidth="1"/>
+    <col min="5" max="5" width="13.44140625" customWidth="1"/>
+    <col min="6" max="6" width="12.88671875" customWidth="1"/>
+    <col min="7" max="7" width="10.77734375" customWidth="1"/>
+    <col min="8" max="8" width="11.109375" customWidth="1"/>
+    <col min="12" max="12" width="13.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15">
+      <c r="A2" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2" s="9"/>
+    </row>
+    <row r="3" spans="1:15">
+      <c r="A3" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15">
+      <c r="A4" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15">
+      <c r="A5" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="E5">
+        <v>8796544376</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15">
+      <c r="A6" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="J6">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15">
+      <c r="A7" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="K7" s="9">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15">
+      <c r="A8" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="L8">
+        <v>98.6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15">
+      <c r="A9" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="M9">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15">
+      <c r="A10" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="N10">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15">
+      <c r="A11" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="M11">
+        <v>93</v>
+      </c>
+      <c r="N11">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15">
+      <c r="A12" s="7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15">
+      <c r="A13" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15">
+      <c r="A14" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15">
+      <c r="A15" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15">
+      <c r="A16" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12">
+      <c r="A17" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12">
+      <c r="A18" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12">
+      <c r="A19" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12">
+      <c r="A20" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12">
+      <c r="A21" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="D21" s="13" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12">
+      <c r="A22" s="7" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12">
+      <c r="A23" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="E23" s="11" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12">
+      <c r="A24" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="E24" s="12" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12">
+      <c r="A25" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12">
+      <c r="A26" s="7" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12">
+      <c r="A27" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="J27" s="11" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12">
+      <c r="A28" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="J28" s="11" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12">
+      <c r="A29" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="K29" s="14" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12">
+      <c r="A30" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="K30" s="11" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12">
+      <c r="A31" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="L31" s="11" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12">
+      <c r="A32" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="L32" s="11" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14">
+      <c r="A33" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="M33" s="11" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14">
+      <c r="A34" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="M34" s="11" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14">
+      <c r="A35" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="M35">
+        <v>94</v>
+      </c>
+      <c r="N35" s="11"/>
+    </row>
+    <row r="36" spans="1:14">
+      <c r="A36" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="N36" s="11" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14">
+      <c r="A37" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="N37" s="11" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14">
+      <c r="A38" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="N38">
+        <v>78</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D4" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>